<commit_message>
benchmark results of WTE without ccs (for tech_selection case)
</commit_message>
<xml_diff>
--- a/dataCaseStudy_WtE/raw_results/technology_selection/Summary.xlsx
+++ b/dataCaseStudy_WtE/raw_results/technology_selection/Summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE169"/>
+  <dimension ref="A1:AE201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17886,6 +17886,3302 @@
       <c r="AE169" t="inlineStr">
         <is>
           <t>dataCaseStudy_WtE\raw_results\technology_selection\20260303011634_dh_1_ctax_250_el_price_400</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="n">
+        <v>16288277.5823403</v>
+      </c>
+      <c r="B170" t="n">
+        <v>298.9250021439932</v>
+      </c>
+      <c r="C170" t="n">
+        <v>0</v>
+      </c>
+      <c r="D170" t="n">
+        <v>345260.7560583042</v>
+      </c>
+      <c r="E170" t="n">
+        <v>0</v>
+      </c>
+      <c r="F170" t="n">
+        <v>345559.6810604482</v>
+      </c>
+      <c r="G170" t="n">
+        <v>0</v>
+      </c>
+      <c r="H170" t="n">
+        <v>155.0546472912404</v>
+      </c>
+      <c r="I170" t="n">
+        <v>-5359875.275964418</v>
+      </c>
+      <c r="J170" t="n">
+        <v>0</v>
+      </c>
+      <c r="K170" t="n">
+        <v>0</v>
+      </c>
+      <c r="L170" t="n">
+        <v>21302438.12259698</v>
+      </c>
+      <c r="M170" t="n">
+        <v>16288277.5823403</v>
+      </c>
+      <c r="N170" t="n">
+        <v>213024.3812259698</v>
+      </c>
+      <c r="O170" t="n">
+        <v>0</v>
+      </c>
+      <c r="P170" t="n">
+        <v>213024.3812259698</v>
+      </c>
+      <c r="Q170" t="n">
+        <v>213024.3812259698</v>
+      </c>
+      <c r="R170" t="n">
+        <v>0</v>
+      </c>
+      <c r="S170" t="n">
+        <v>0</v>
+      </c>
+      <c r="T170" t="n">
+        <v>0</v>
+      </c>
+      <c r="U170" t="n">
+        <v>0</v>
+      </c>
+      <c r="V170" t="n">
+        <v>2.365000009536743</v>
+      </c>
+      <c r="W170" t="n">
+        <v>16288277.5823403</v>
+      </c>
+      <c r="X170" t="n">
+        <v>16288277.5823403</v>
+      </c>
+      <c r="Y170" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z170" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA170" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB170" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC170" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD170" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_100_el_price_50</t>
+        </is>
+      </c>
+      <c r="AE170" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\technology_selection\20260303183248_dh_0.5_ctax_100_el_price_50</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="n">
+        <v>10925191.3762467</v>
+      </c>
+      <c r="B171" t="n">
+        <v>298.9250021439932</v>
+      </c>
+      <c r="C171" t="n">
+        <v>0</v>
+      </c>
+      <c r="D171" t="n">
+        <v>345260.7560583042</v>
+      </c>
+      <c r="E171" t="n">
+        <v>0</v>
+      </c>
+      <c r="F171" t="n">
+        <v>345559.6810604482</v>
+      </c>
+      <c r="G171" t="n">
+        <v>0</v>
+      </c>
+      <c r="H171" t="n">
+        <v>16256.29726210878</v>
+      </c>
+      <c r="I171" t="n">
+        <v>-10746509.54938219</v>
+      </c>
+      <c r="J171" t="n">
+        <v>0</v>
+      </c>
+      <c r="K171" t="n">
+        <v>0</v>
+      </c>
+      <c r="L171" t="n">
+        <v>21309884.94730634</v>
+      </c>
+      <c r="M171" t="n">
+        <v>10925191.3762467</v>
+      </c>
+      <c r="N171" t="n">
+        <v>213098.8494730633</v>
+      </c>
+      <c r="O171" t="n">
+        <v>0</v>
+      </c>
+      <c r="P171" t="n">
+        <v>213098.8494730633</v>
+      </c>
+      <c r="Q171" t="n">
+        <v>213098.8494730633</v>
+      </c>
+      <c r="R171" t="n">
+        <v>0</v>
+      </c>
+      <c r="S171" t="n">
+        <v>0</v>
+      </c>
+      <c r="T171" t="n">
+        <v>0</v>
+      </c>
+      <c r="U171" t="n">
+        <v>0</v>
+      </c>
+      <c r="V171" t="n">
+        <v>1.797000169754028</v>
+      </c>
+      <c r="W171" t="n">
+        <v>10925191.37624663</v>
+      </c>
+      <c r="X171" t="n">
+        <v>10925191.3762467</v>
+      </c>
+      <c r="Y171" t="n">
+        <v>6.705522537231445e-08</v>
+      </c>
+      <c r="Z171" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA171" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB171" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC171" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD171" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_100_el_price_100</t>
+        </is>
+      </c>
+      <c r="AE171" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\technology_selection\20260303183508_dh_0.5_ctax_100_el_price_100</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="n">
+        <v>5509548.414125333</v>
+      </c>
+      <c r="B172" t="n">
+        <v>298.9250021439932</v>
+      </c>
+      <c r="C172" t="n">
+        <v>0</v>
+      </c>
+      <c r="D172" t="n">
+        <v>345260.7560583042</v>
+      </c>
+      <c r="E172" t="n">
+        <v>0</v>
+      </c>
+      <c r="F172" t="n">
+        <v>345559.6810604482</v>
+      </c>
+      <c r="G172" t="n">
+        <v>0</v>
+      </c>
+      <c r="H172" t="n">
+        <v>251892.889191721</v>
+      </c>
+      <c r="I172" t="n">
+        <v>-16506771.02720062</v>
+      </c>
+      <c r="J172" t="n">
+        <v>0</v>
+      </c>
+      <c r="K172" t="n">
+        <v>0</v>
+      </c>
+      <c r="L172" t="n">
+        <v>21418866.87107379</v>
+      </c>
+      <c r="M172" t="n">
+        <v>5509548.414125333</v>
+      </c>
+      <c r="N172" t="n">
+        <v>214188.6687107377</v>
+      </c>
+      <c r="O172" t="n">
+        <v>0</v>
+      </c>
+      <c r="P172" t="n">
+        <v>214188.6687107377</v>
+      </c>
+      <c r="Q172" t="n">
+        <v>214188.6687107378</v>
+      </c>
+      <c r="R172" t="n">
+        <v>0</v>
+      </c>
+      <c r="S172" t="n">
+        <v>0</v>
+      </c>
+      <c r="T172" t="n">
+        <v>0</v>
+      </c>
+      <c r="U172" t="n">
+        <v>0</v>
+      </c>
+      <c r="V172" t="n">
+        <v>1.769000053405762</v>
+      </c>
+      <c r="W172" t="n">
+        <v>5509548.414125187</v>
+      </c>
+      <c r="X172" t="n">
+        <v>5509548.414125333</v>
+      </c>
+      <c r="Y172" t="n">
+        <v>1.452863216400146e-07</v>
+      </c>
+      <c r="Z172" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA172" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB172" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC172" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD172" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_100_el_price_150</t>
+        </is>
+      </c>
+      <c r="AE172" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\technology_selection\20260303183718_dh_0.5_ctax_100_el_price_150</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="n">
+        <v>-111513.2904379889</v>
+      </c>
+      <c r="B173" t="n">
+        <v>298.9250021439932</v>
+      </c>
+      <c r="C173" t="n">
+        <v>0</v>
+      </c>
+      <c r="D173" t="n">
+        <v>345260.7560583042</v>
+      </c>
+      <c r="E173" t="n">
+        <v>0</v>
+      </c>
+      <c r="F173" t="n">
+        <v>345559.6810604482</v>
+      </c>
+      <c r="G173" t="n">
+        <v>0</v>
+      </c>
+      <c r="H173" t="n">
+        <v>876781.4848603355</v>
+      </c>
+      <c r="I173" t="n">
+        <v>-23041732.30292929</v>
+      </c>
+      <c r="J173" t="n">
+        <v>0</v>
+      </c>
+      <c r="K173" t="n">
+        <v>0</v>
+      </c>
+      <c r="L173" t="n">
+        <v>21707877.84657052</v>
+      </c>
+      <c r="M173" t="n">
+        <v>-111513.2904379889</v>
+      </c>
+      <c r="N173" t="n">
+        <v>217078.7784657051</v>
+      </c>
+      <c r="O173" t="n">
+        <v>0</v>
+      </c>
+      <c r="P173" t="n">
+        <v>217078.7784657051</v>
+      </c>
+      <c r="Q173" t="n">
+        <v>217078.7784657051</v>
+      </c>
+      <c r="R173" t="n">
+        <v>0</v>
+      </c>
+      <c r="S173" t="n">
+        <v>0</v>
+      </c>
+      <c r="T173" t="n">
+        <v>0</v>
+      </c>
+      <c r="U173" t="n">
+        <v>0</v>
+      </c>
+      <c r="V173" t="n">
+        <v>1.784999847412109</v>
+      </c>
+      <c r="W173" t="n">
+        <v>-111513.2904379889</v>
+      </c>
+      <c r="X173" t="n">
+        <v>-111513.2904379889</v>
+      </c>
+      <c r="Y173" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z173" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA173" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB173" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC173" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD173" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_100_el_price_200</t>
+        </is>
+      </c>
+      <c r="AE173" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\technology_selection\20260303183937_dh_0.5_ctax_100_el_price_200</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="n">
+        <v>-6012420.672834076</v>
+      </c>
+      <c r="B174" t="n">
+        <v>298.9250021439932</v>
+      </c>
+      <c r="C174" t="n">
+        <v>0</v>
+      </c>
+      <c r="D174" t="n">
+        <v>345260.7560583042</v>
+      </c>
+      <c r="E174" t="n">
+        <v>0</v>
+      </c>
+      <c r="F174" t="n">
+        <v>345559.6810604482</v>
+      </c>
+      <c r="G174" t="n">
+        <v>0</v>
+      </c>
+      <c r="H174" t="n">
+        <v>1647033.57777678</v>
+      </c>
+      <c r="I174" t="n">
+        <v>-30069133.37121568</v>
+      </c>
+      <c r="J174" t="n">
+        <v>0</v>
+      </c>
+      <c r="K174" t="n">
+        <v>0</v>
+      </c>
+      <c r="L174" t="n">
+        <v>22064119.43954438</v>
+      </c>
+      <c r="M174" t="n">
+        <v>-6012420.672834076</v>
+      </c>
+      <c r="N174" t="n">
+        <v>220641.1943954437</v>
+      </c>
+      <c r="O174" t="n">
+        <v>0</v>
+      </c>
+      <c r="P174" t="n">
+        <v>220641.1943954437</v>
+      </c>
+      <c r="Q174" t="n">
+        <v>220641.1943954437</v>
+      </c>
+      <c r="R174" t="n">
+        <v>0</v>
+      </c>
+      <c r="S174" t="n">
+        <v>0</v>
+      </c>
+      <c r="T174" t="n">
+        <v>0</v>
+      </c>
+      <c r="U174" t="n">
+        <v>0</v>
+      </c>
+      <c r="V174" t="n">
+        <v>2.006999969482422</v>
+      </c>
+      <c r="W174" t="n">
+        <v>-6012420.672834076</v>
+      </c>
+      <c r="X174" t="n">
+        <v>-6012420.672834076</v>
+      </c>
+      <c r="Y174" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z174" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA174" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB174" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC174" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD174" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_100_el_price_250</t>
+        </is>
+      </c>
+      <c r="AE174" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\technology_selection\20260303184145_dh_0.5_ctax_100_el_price_250</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="n">
+        <v>-12074800.50869442</v>
+      </c>
+      <c r="B175" t="n">
+        <v>298.9250021439932</v>
+      </c>
+      <c r="C175" t="n">
+        <v>0</v>
+      </c>
+      <c r="D175" t="n">
+        <v>345260.7560583042</v>
+      </c>
+      <c r="E175" t="n">
+        <v>0</v>
+      </c>
+      <c r="F175" t="n">
+        <v>345559.6810604482</v>
+      </c>
+      <c r="G175" t="n">
+        <v>0</v>
+      </c>
+      <c r="H175" t="n">
+        <v>1943719.78314256</v>
+      </c>
+      <c r="I175" t="n">
+        <v>-36565416.78242347</v>
+      </c>
+      <c r="J175" t="n">
+        <v>0</v>
+      </c>
+      <c r="K175" t="n">
+        <v>0</v>
+      </c>
+      <c r="L175" t="n">
+        <v>22201336.80952604</v>
+      </c>
+      <c r="M175" t="n">
+        <v>-12074800.50869442</v>
+      </c>
+      <c r="N175" t="n">
+        <v>222013.3680952604</v>
+      </c>
+      <c r="O175" t="n">
+        <v>0</v>
+      </c>
+      <c r="P175" t="n">
+        <v>222013.3680952604</v>
+      </c>
+      <c r="Q175" t="n">
+        <v>222013.3680952604</v>
+      </c>
+      <c r="R175" t="n">
+        <v>0</v>
+      </c>
+      <c r="S175" t="n">
+        <v>0</v>
+      </c>
+      <c r="T175" t="n">
+        <v>0</v>
+      </c>
+      <c r="U175" t="n">
+        <v>0</v>
+      </c>
+      <c r="V175" t="n">
+        <v>2.183000087738037</v>
+      </c>
+      <c r="W175" t="n">
+        <v>-12074800.50869448</v>
+      </c>
+      <c r="X175" t="n">
+        <v>-12074800.50869442</v>
+      </c>
+      <c r="Y175" t="n">
+        <v>5.587935447692871e-08</v>
+      </c>
+      <c r="Z175" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA175" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB175" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC175" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD175" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_100_el_price_300</t>
+        </is>
+      </c>
+      <c r="AE175" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\technology_selection\20260303184409_dh_0.5_ctax_100_el_price_300</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="n">
+        <v>-18183808.08255287</v>
+      </c>
+      <c r="B176" t="n">
+        <v>298.9250021439932</v>
+      </c>
+      <c r="C176" t="n">
+        <v>0</v>
+      </c>
+      <c r="D176" t="n">
+        <v>345260.7560583042</v>
+      </c>
+      <c r="E176" t="n">
+        <v>0</v>
+      </c>
+      <c r="F176" t="n">
+        <v>345559.6810604482</v>
+      </c>
+      <c r="G176" t="n">
+        <v>0</v>
+      </c>
+      <c r="H176" t="n">
+        <v>2061813.094625738</v>
+      </c>
+      <c r="I176" t="n">
+        <v>-42847135.82432608</v>
+      </c>
+      <c r="J176" t="n">
+        <v>0</v>
+      </c>
+      <c r="K176" t="n">
+        <v>0</v>
+      </c>
+      <c r="L176" t="n">
+        <v>22255954.96608701</v>
+      </c>
+      <c r="M176" t="n">
+        <v>-18183808.08255287</v>
+      </c>
+      <c r="N176" t="n">
+        <v>222559.5496608701</v>
+      </c>
+      <c r="O176" t="n">
+        <v>0</v>
+      </c>
+      <c r="P176" t="n">
+        <v>222559.5496608701</v>
+      </c>
+      <c r="Q176" t="n">
+        <v>222559.5496608701</v>
+      </c>
+      <c r="R176" t="n">
+        <v>0</v>
+      </c>
+      <c r="S176" t="n">
+        <v>0</v>
+      </c>
+      <c r="T176" t="n">
+        <v>0</v>
+      </c>
+      <c r="U176" t="n">
+        <v>0</v>
+      </c>
+      <c r="V176" t="n">
+        <v>1.847000122070312</v>
+      </c>
+      <c r="W176" t="n">
+        <v>-18183808.08255288</v>
+      </c>
+      <c r="X176" t="n">
+        <v>-18183808.08255287</v>
+      </c>
+      <c r="Y176" t="n">
+        <v>7.450580596923828e-09</v>
+      </c>
+      <c r="Z176" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA176" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB176" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC176" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD176" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_100_el_price_350</t>
+        </is>
+      </c>
+      <c r="AE176" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\technology_selection\20260303184703_dh_0.5_ctax_100_el_price_350</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="n">
+        <v>-24308846.4052638</v>
+      </c>
+      <c r="B177" t="n">
+        <v>298.9250021439932</v>
+      </c>
+      <c r="C177" t="n">
+        <v>0</v>
+      </c>
+      <c r="D177" t="n">
+        <v>345260.7560583042</v>
+      </c>
+      <c r="E177" t="n">
+        <v>0</v>
+      </c>
+      <c r="F177" t="n">
+        <v>345559.6810604482</v>
+      </c>
+      <c r="G177" t="n">
+        <v>0</v>
+      </c>
+      <c r="H177" t="n">
+        <v>2094069.069521546</v>
+      </c>
+      <c r="I177" t="n">
+        <v>-49019348.51032212</v>
+      </c>
+      <c r="J177" t="n">
+        <v>0</v>
+      </c>
+      <c r="K177" t="n">
+        <v>0</v>
+      </c>
+      <c r="L177" t="n">
+        <v>22270873.35447633</v>
+      </c>
+      <c r="M177" t="n">
+        <v>-24308846.4052638</v>
+      </c>
+      <c r="N177" t="n">
+        <v>222708.7335447632</v>
+      </c>
+      <c r="O177" t="n">
+        <v>0</v>
+      </c>
+      <c r="P177" t="n">
+        <v>222708.7335447632</v>
+      </c>
+      <c r="Q177" t="n">
+        <v>222708.7335447632</v>
+      </c>
+      <c r="R177" t="n">
+        <v>0</v>
+      </c>
+      <c r="S177" t="n">
+        <v>0</v>
+      </c>
+      <c r="T177" t="n">
+        <v>0</v>
+      </c>
+      <c r="U177" t="n">
+        <v>0</v>
+      </c>
+      <c r="V177" t="n">
+        <v>1.91700005531311</v>
+      </c>
+      <c r="W177" t="n">
+        <v>-24308846.40526384</v>
+      </c>
+      <c r="X177" t="n">
+        <v>-24308846.4052638</v>
+      </c>
+      <c r="Y177" t="n">
+        <v>3.725290298461914e-08</v>
+      </c>
+      <c r="Z177" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA177" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB177" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC177" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD177" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_100_el_price_400</t>
+        </is>
+      </c>
+      <c r="AE177" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\technology_selection\20260303184935_dh_0.5_ctax_100_el_price_400</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="n">
+        <v>26939496.6436388</v>
+      </c>
+      <c r="B178" t="n">
+        <v>298.9250021439932</v>
+      </c>
+      <c r="C178" t="n">
+        <v>0</v>
+      </c>
+      <c r="D178" t="n">
+        <v>345260.7560583042</v>
+      </c>
+      <c r="E178" t="n">
+        <v>0</v>
+      </c>
+      <c r="F178" t="n">
+        <v>345559.6810604482</v>
+      </c>
+      <c r="G178" t="n">
+        <v>0</v>
+      </c>
+      <c r="H178" t="n">
+        <v>155.0546472912404</v>
+      </c>
+      <c r="I178" t="n">
+        <v>-5359875.275964418</v>
+      </c>
+      <c r="J178" t="n">
+        <v>0</v>
+      </c>
+      <c r="K178" t="n">
+        <v>0</v>
+      </c>
+      <c r="L178" t="n">
+        <v>31953657.18389548</v>
+      </c>
+      <c r="M178" t="n">
+        <v>26939496.6436388</v>
+      </c>
+      <c r="N178" t="n">
+        <v>213024.3812259698</v>
+      </c>
+      <c r="O178" t="n">
+        <v>0</v>
+      </c>
+      <c r="P178" t="n">
+        <v>213024.3812259698</v>
+      </c>
+      <c r="Q178" t="n">
+        <v>213024.3812259698</v>
+      </c>
+      <c r="R178" t="n">
+        <v>0</v>
+      </c>
+      <c r="S178" t="n">
+        <v>0</v>
+      </c>
+      <c r="T178" t="n">
+        <v>0</v>
+      </c>
+      <c r="U178" t="n">
+        <v>0</v>
+      </c>
+      <c r="V178" t="n">
+        <v>1.920000076293945</v>
+      </c>
+      <c r="W178" t="n">
+        <v>26939496.6436388</v>
+      </c>
+      <c r="X178" t="n">
+        <v>26939496.6436388</v>
+      </c>
+      <c r="Y178" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z178" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA178" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB178" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC178" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD178" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_150_el_price_50</t>
+        </is>
+      </c>
+      <c r="AE178" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\technology_selection\20260303185208_dh_0.5_ctax_150_el_price_50</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="n">
+        <v>21579106.17715645</v>
+      </c>
+      <c r="B179" t="n">
+        <v>298.9250021439932</v>
+      </c>
+      <c r="C179" t="n">
+        <v>0</v>
+      </c>
+      <c r="D179" t="n">
+        <v>345260.7560583042</v>
+      </c>
+      <c r="E179" t="n">
+        <v>0</v>
+      </c>
+      <c r="F179" t="n">
+        <v>345559.6810604482</v>
+      </c>
+      <c r="G179" t="n">
+        <v>0</v>
+      </c>
+      <c r="H179" t="n">
+        <v>7417.093733416082</v>
+      </c>
+      <c r="I179" t="n">
+        <v>-10732565.82114889</v>
+      </c>
+      <c r="J179" t="n">
+        <v>0</v>
+      </c>
+      <c r="K179" t="n">
+        <v>0</v>
+      </c>
+      <c r="L179" t="n">
+        <v>31958695.22351148</v>
+      </c>
+      <c r="M179" t="n">
+        <v>21579106.17715645</v>
+      </c>
+      <c r="N179" t="n">
+        <v>213057.9681567431</v>
+      </c>
+      <c r="O179" t="n">
+        <v>0</v>
+      </c>
+      <c r="P179" t="n">
+        <v>213057.9681567431</v>
+      </c>
+      <c r="Q179" t="n">
+        <v>213057.9681567431</v>
+      </c>
+      <c r="R179" t="n">
+        <v>0</v>
+      </c>
+      <c r="S179" t="n">
+        <v>0</v>
+      </c>
+      <c r="T179" t="n">
+        <v>0</v>
+      </c>
+      <c r="U179" t="n">
+        <v>0</v>
+      </c>
+      <c r="V179" t="n">
+        <v>1.688999891281128</v>
+      </c>
+      <c r="W179" t="n">
+        <v>21579106.17715633</v>
+      </c>
+      <c r="X179" t="n">
+        <v>21579106.17715645</v>
+      </c>
+      <c r="Y179" t="n">
+        <v>1.229345798492432e-07</v>
+      </c>
+      <c r="Z179" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA179" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB179" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC179" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD179" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_150_el_price_100</t>
+        </is>
+      </c>
+      <c r="AE179" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\technology_selection\20260303185357_dh_0.5_ctax_150_el_price_100</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="n">
+        <v>16197266.25525175</v>
+      </c>
+      <c r="B180" t="n">
+        <v>298.9250021439932</v>
+      </c>
+      <c r="C180" t="n">
+        <v>0</v>
+      </c>
+      <c r="D180" t="n">
+        <v>345260.7560583042</v>
+      </c>
+      <c r="E180" t="n">
+        <v>0</v>
+      </c>
+      <c r="F180" t="n">
+        <v>345559.6810604482</v>
+      </c>
+      <c r="G180" t="n">
+        <v>0</v>
+      </c>
+      <c r="H180" t="n">
+        <v>84354.75926208599</v>
+      </c>
+      <c r="I180" t="n">
+        <v>-16244718.91404278</v>
+      </c>
+      <c r="J180" t="n">
+        <v>0</v>
+      </c>
+      <c r="K180" t="n">
+        <v>0</v>
+      </c>
+      <c r="L180" t="n">
+        <v>32012070.728972</v>
+      </c>
+      <c r="M180" t="n">
+        <v>16197266.25525175</v>
+      </c>
+      <c r="N180" t="n">
+        <v>213413.8048598132</v>
+      </c>
+      <c r="O180" t="n">
+        <v>0</v>
+      </c>
+      <c r="P180" t="n">
+        <v>213413.8048598132</v>
+      </c>
+      <c r="Q180" t="n">
+        <v>213413.8048598132</v>
+      </c>
+      <c r="R180" t="n">
+        <v>0</v>
+      </c>
+      <c r="S180" t="n">
+        <v>0</v>
+      </c>
+      <c r="T180" t="n">
+        <v>0</v>
+      </c>
+      <c r="U180" t="n">
+        <v>0</v>
+      </c>
+      <c r="V180" t="n">
+        <v>1.884000062942505</v>
+      </c>
+      <c r="W180" t="n">
+        <v>16197266.25525155</v>
+      </c>
+      <c r="X180" t="n">
+        <v>16197266.25525175</v>
+      </c>
+      <c r="Y180" t="n">
+        <v>2.048909664154053e-07</v>
+      </c>
+      <c r="Z180" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA180" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB180" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC180" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD180" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_150_el_price_150</t>
+        </is>
+      </c>
+      <c r="AE180" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\technology_selection\20260303185642_dh_0.5_ctax_150_el_price_150</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="n">
+        <v>10693572.4615687</v>
+      </c>
+      <c r="B181" t="n">
+        <v>298.9250021439932</v>
+      </c>
+      <c r="C181" t="n">
+        <v>0</v>
+      </c>
+      <c r="D181" t="n">
+        <v>345260.7560583042</v>
+      </c>
+      <c r="E181" t="n">
+        <v>0</v>
+      </c>
+      <c r="F181" t="n">
+        <v>345559.6810604482</v>
+      </c>
+      <c r="G181" t="n">
+        <v>0</v>
+      </c>
+      <c r="H181" t="n">
+        <v>475452.0461187353</v>
+      </c>
+      <c r="I181" t="n">
+        <v>-22410833.73733928</v>
+      </c>
+      <c r="J181" t="n">
+        <v>0</v>
+      </c>
+      <c r="K181" t="n">
+        <v>0</v>
+      </c>
+      <c r="L181" t="n">
+        <v>32283394.4717288</v>
+      </c>
+      <c r="M181" t="n">
+        <v>10693572.4615687</v>
+      </c>
+      <c r="N181" t="n">
+        <v>215222.6298115252</v>
+      </c>
+      <c r="O181" t="n">
+        <v>0</v>
+      </c>
+      <c r="P181" t="n">
+        <v>215222.6298115252</v>
+      </c>
+      <c r="Q181" t="n">
+        <v>215222.6298115252</v>
+      </c>
+      <c r="R181" t="n">
+        <v>0</v>
+      </c>
+      <c r="S181" t="n">
+        <v>0</v>
+      </c>
+      <c r="T181" t="n">
+        <v>0</v>
+      </c>
+      <c r="U181" t="n">
+        <v>0</v>
+      </c>
+      <c r="V181" t="n">
+        <v>1.677000045776367</v>
+      </c>
+      <c r="W181" t="n">
+        <v>10693572.46156869</v>
+      </c>
+      <c r="X181" t="n">
+        <v>10693572.4615687</v>
+      </c>
+      <c r="Y181" t="n">
+        <v>7.450580596923828e-09</v>
+      </c>
+      <c r="Z181" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA181" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB181" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC181" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD181" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_150_el_price_200</t>
+        </is>
+      </c>
+      <c r="AE181" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\technology_selection\20260303185832_dh_0.5_ctax_150_el_price_200</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="n">
+        <v>4964457.577288527</v>
+      </c>
+      <c r="B182" t="n">
+        <v>298.9250021439932</v>
+      </c>
+      <c r="C182" t="n">
+        <v>0</v>
+      </c>
+      <c r="D182" t="n">
+        <v>345260.7560583042</v>
+      </c>
+      <c r="E182" t="n">
+        <v>0</v>
+      </c>
+      <c r="F182" t="n">
+        <v>345559.6810604482</v>
+      </c>
+      <c r="G182" t="n">
+        <v>0</v>
+      </c>
+      <c r="H182" t="n">
+        <v>1144370.416970436</v>
+      </c>
+      <c r="I182" t="n">
+        <v>-29272929.11224952</v>
+      </c>
+      <c r="J182" t="n">
+        <v>0</v>
+      </c>
+      <c r="K182" t="n">
+        <v>0</v>
+      </c>
+      <c r="L182" t="n">
+        <v>32747456.59150717</v>
+      </c>
+      <c r="M182" t="n">
+        <v>4964457.577288527</v>
+      </c>
+      <c r="N182" t="n">
+        <v>218316.3772767143</v>
+      </c>
+      <c r="O182" t="n">
+        <v>0</v>
+      </c>
+      <c r="P182" t="n">
+        <v>218316.3772767143</v>
+      </c>
+      <c r="Q182" t="n">
+        <v>218316.3772767144</v>
+      </c>
+      <c r="R182" t="n">
+        <v>0</v>
+      </c>
+      <c r="S182" t="n">
+        <v>0</v>
+      </c>
+      <c r="T182" t="n">
+        <v>0</v>
+      </c>
+      <c r="U182" t="n">
+        <v>0</v>
+      </c>
+      <c r="V182" t="n">
+        <v>1.808000087738037</v>
+      </c>
+      <c r="W182" t="n">
+        <v>4964457.577288481</v>
+      </c>
+      <c r="X182" t="n">
+        <v>4964457.577288527</v>
+      </c>
+      <c r="Y182" t="n">
+        <v>4.563480615615845e-08</v>
+      </c>
+      <c r="Z182" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA182" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB182" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC182" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD182" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_150_el_price_250</t>
+        </is>
+      </c>
+      <c r="AE182" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\technology_selection\20260303190128_dh_0.5_ctax_150_el_price_250</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="n">
+        <v>-996204.8174847178</v>
+      </c>
+      <c r="B183" t="n">
+        <v>298.9250021439932</v>
+      </c>
+      <c r="C183" t="n">
+        <v>0</v>
+      </c>
+      <c r="D183" t="n">
+        <v>345260.7560583042</v>
+      </c>
+      <c r="E183" t="n">
+        <v>0</v>
+      </c>
+      <c r="F183" t="n">
+        <v>345559.6810604482</v>
+      </c>
+      <c r="G183" t="n">
+        <v>0</v>
+      </c>
+      <c r="H183" t="n">
+        <v>1709345.297483764</v>
+      </c>
+      <c r="I183" t="n">
+        <v>-36190517.71089222</v>
+      </c>
+      <c r="J183" t="n">
+        <v>0</v>
+      </c>
+      <c r="K183" t="n">
+        <v>0</v>
+      </c>
+      <c r="L183" t="n">
+        <v>33139407.91486328</v>
+      </c>
+      <c r="M183" t="n">
+        <v>-996204.8174847178</v>
+      </c>
+      <c r="N183" t="n">
+        <v>220929.3860990884</v>
+      </c>
+      <c r="O183" t="n">
+        <v>0</v>
+      </c>
+      <c r="P183" t="n">
+        <v>220929.3860990884</v>
+      </c>
+      <c r="Q183" t="n">
+        <v>220929.3860990885</v>
+      </c>
+      <c r="R183" t="n">
+        <v>0</v>
+      </c>
+      <c r="S183" t="n">
+        <v>0</v>
+      </c>
+      <c r="T183" t="n">
+        <v>0</v>
+      </c>
+      <c r="U183" t="n">
+        <v>0</v>
+      </c>
+      <c r="V183" t="n">
+        <v>1.611999988555908</v>
+      </c>
+      <c r="W183" t="n">
+        <v>-996204.8174847807</v>
+      </c>
+      <c r="X183" t="n">
+        <v>-996204.8174847178</v>
+      </c>
+      <c r="Y183" t="n">
+        <v>6.28642737865448e-08</v>
+      </c>
+      <c r="Z183" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA183" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB183" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC183" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD183" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_150_el_price_300</t>
+        </is>
+      </c>
+      <c r="AE183" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\technology_selection\20260303190316_dh_0.5_ctax_150_el_price_300</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="n">
+        <v>-7068393.308029361</v>
+      </c>
+      <c r="B184" t="n">
+        <v>298.9250021439932</v>
+      </c>
+      <c r="C184" t="n">
+        <v>0</v>
+      </c>
+      <c r="D184" t="n">
+        <v>345260.7560583042</v>
+      </c>
+      <c r="E184" t="n">
+        <v>0</v>
+      </c>
+      <c r="F184" t="n">
+        <v>345559.6810604482</v>
+      </c>
+      <c r="G184" t="n">
+        <v>0</v>
+      </c>
+      <c r="H184" t="n">
+        <v>1949433.947739025</v>
+      </c>
+      <c r="I184" t="n">
+        <v>-42669356.35280671</v>
+      </c>
+      <c r="J184" t="n">
+        <v>0</v>
+      </c>
+      <c r="K184" t="n">
+        <v>0</v>
+      </c>
+      <c r="L184" t="n">
+        <v>33305969.41597787</v>
+      </c>
+      <c r="M184" t="n">
+        <v>-7068393.308029361</v>
+      </c>
+      <c r="N184" t="n">
+        <v>222039.7961065191</v>
+      </c>
+      <c r="O184" t="n">
+        <v>0</v>
+      </c>
+      <c r="P184" t="n">
+        <v>222039.7961065191</v>
+      </c>
+      <c r="Q184" t="n">
+        <v>222039.7961065191</v>
+      </c>
+      <c r="R184" t="n">
+        <v>0</v>
+      </c>
+      <c r="S184" t="n">
+        <v>0</v>
+      </c>
+      <c r="T184" t="n">
+        <v>0</v>
+      </c>
+      <c r="U184" t="n">
+        <v>0</v>
+      </c>
+      <c r="V184" t="n">
+        <v>1.636999845504761</v>
+      </c>
+      <c r="W184" t="n">
+        <v>-7068393.308029442</v>
+      </c>
+      <c r="X184" t="n">
+        <v>-7068393.308029361</v>
+      </c>
+      <c r="Y184" t="n">
+        <v>8.102506399154663e-08</v>
+      </c>
+      <c r="Z184" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA184" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB184" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC184" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD184" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_150_el_price_350</t>
+        </is>
+      </c>
+      <c r="AE184" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\technology_selection\20260303190503_dh_0.5_ctax_150_el_price_350</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="n">
+        <v>-13176895.49283775</v>
+      </c>
+      <c r="B185" t="n">
+        <v>298.9250021439932</v>
+      </c>
+      <c r="C185" t="n">
+        <v>0</v>
+      </c>
+      <c r="D185" t="n">
+        <v>345260.7560583042</v>
+      </c>
+      <c r="E185" t="n">
+        <v>0</v>
+      </c>
+      <c r="F185" t="n">
+        <v>345559.6810604482</v>
+      </c>
+      <c r="G185" t="n">
+        <v>0</v>
+      </c>
+      <c r="H185" t="n">
+        <v>2057857.107913282</v>
+      </c>
+      <c r="I185" t="n">
+        <v>-48961500.26516025</v>
+      </c>
+      <c r="J185" t="n">
+        <v>0</v>
+      </c>
+      <c r="K185" t="n">
+        <v>0</v>
+      </c>
+      <c r="L185" t="n">
+        <v>33381187.98334876</v>
+      </c>
+      <c r="M185" t="n">
+        <v>-13176895.49283775</v>
+      </c>
+      <c r="N185" t="n">
+        <v>222541.253222325</v>
+      </c>
+      <c r="O185" t="n">
+        <v>0</v>
+      </c>
+      <c r="P185" t="n">
+        <v>222541.253222325</v>
+      </c>
+      <c r="Q185" t="n">
+        <v>222541.253222325</v>
+      </c>
+      <c r="R185" t="n">
+        <v>0</v>
+      </c>
+      <c r="S185" t="n">
+        <v>0</v>
+      </c>
+      <c r="T185" t="n">
+        <v>0</v>
+      </c>
+      <c r="U185" t="n">
+        <v>0</v>
+      </c>
+      <c r="V185" t="n">
+        <v>1.580999851226807</v>
+      </c>
+      <c r="W185" t="n">
+        <v>-13176895.49283778</v>
+      </c>
+      <c r="X185" t="n">
+        <v>-13176895.49283775</v>
+      </c>
+      <c r="Y185" t="n">
+        <v>3.352761268615723e-08</v>
+      </c>
+      <c r="Z185" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA185" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB185" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC185" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD185" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_150_el_price_400</t>
+        </is>
+      </c>
+      <c r="AE185" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\technology_selection\20260303190813_dh_0.5_ctax_150_el_price_400</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="n">
+        <v>37590715.70493729</v>
+      </c>
+      <c r="B186" t="n">
+        <v>298.9250021439932</v>
+      </c>
+      <c r="C186" t="n">
+        <v>0</v>
+      </c>
+      <c r="D186" t="n">
+        <v>345260.7560583042</v>
+      </c>
+      <c r="E186" t="n">
+        <v>0</v>
+      </c>
+      <c r="F186" t="n">
+        <v>345559.6810604482</v>
+      </c>
+      <c r="G186" t="n">
+        <v>0</v>
+      </c>
+      <c r="H186" t="n">
+        <v>155.0546472912404</v>
+      </c>
+      <c r="I186" t="n">
+        <v>-5359875.275964418</v>
+      </c>
+      <c r="J186" t="n">
+        <v>0</v>
+      </c>
+      <c r="K186" t="n">
+        <v>0</v>
+      </c>
+      <c r="L186" t="n">
+        <v>42604876.24519397</v>
+      </c>
+      <c r="M186" t="n">
+        <v>37590715.70493729</v>
+      </c>
+      <c r="N186" t="n">
+        <v>213024.3812259698</v>
+      </c>
+      <c r="O186" t="n">
+        <v>0</v>
+      </c>
+      <c r="P186" t="n">
+        <v>213024.3812259698</v>
+      </c>
+      <c r="Q186" t="n">
+        <v>213024.3812259698</v>
+      </c>
+      <c r="R186" t="n">
+        <v>0</v>
+      </c>
+      <c r="S186" t="n">
+        <v>0</v>
+      </c>
+      <c r="T186" t="n">
+        <v>0</v>
+      </c>
+      <c r="U186" t="n">
+        <v>0</v>
+      </c>
+      <c r="V186" t="n">
+        <v>1.616000175476074</v>
+      </c>
+      <c r="W186" t="n">
+        <v>37590715.70493698</v>
+      </c>
+      <c r="X186" t="n">
+        <v>37590715.70493729</v>
+      </c>
+      <c r="Y186" t="n">
+        <v>3.05473804473877e-07</v>
+      </c>
+      <c r="Z186" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA186" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB186" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC186" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD186" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_200_el_price_50</t>
+        </is>
+      </c>
+      <c r="AE186" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\technology_selection\20260303190959_dh_0.5_ctax_200_el_price_50</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="n">
+        <v>32230840.42897287</v>
+      </c>
+      <c r="B187" t="n">
+        <v>298.9250021439932</v>
+      </c>
+      <c r="C187" t="n">
+        <v>0</v>
+      </c>
+      <c r="D187" t="n">
+        <v>345260.7560583042</v>
+      </c>
+      <c r="E187" t="n">
+        <v>0</v>
+      </c>
+      <c r="F187" t="n">
+        <v>345559.6810604482</v>
+      </c>
+      <c r="G187" t="n">
+        <v>0</v>
+      </c>
+      <c r="H187" t="n">
+        <v>155.0546472912404</v>
+      </c>
+      <c r="I187" t="n">
+        <v>-10719750.55192884</v>
+      </c>
+      <c r="J187" t="n">
+        <v>0</v>
+      </c>
+      <c r="K187" t="n">
+        <v>0</v>
+      </c>
+      <c r="L187" t="n">
+        <v>42604876.24519397</v>
+      </c>
+      <c r="M187" t="n">
+        <v>32230840.42897287</v>
+      </c>
+      <c r="N187" t="n">
+        <v>213024.3812259698</v>
+      </c>
+      <c r="O187" t="n">
+        <v>0</v>
+      </c>
+      <c r="P187" t="n">
+        <v>213024.3812259698</v>
+      </c>
+      <c r="Q187" t="n">
+        <v>213024.3812259698</v>
+      </c>
+      <c r="R187" t="n">
+        <v>0</v>
+      </c>
+      <c r="S187" t="n">
+        <v>0</v>
+      </c>
+      <c r="T187" t="n">
+        <v>0</v>
+      </c>
+      <c r="U187" t="n">
+        <v>0</v>
+      </c>
+      <c r="V187" t="n">
+        <v>1.601999998092651</v>
+      </c>
+      <c r="W187" t="n">
+        <v>32230840.42897287</v>
+      </c>
+      <c r="X187" t="n">
+        <v>32230840.42897287</v>
+      </c>
+      <c r="Y187" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z187" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA187" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB187" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC187" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD187" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_200_el_price_100</t>
+        </is>
+      </c>
+      <c r="AE187" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\technology_selection\20260303191147_dh_0.5_ctax_200_el_price_100</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="n">
+        <v>26859881.41254083</v>
+      </c>
+      <c r="B188" t="n">
+        <v>298.9250021439932</v>
+      </c>
+      <c r="C188" t="n">
+        <v>0</v>
+      </c>
+      <c r="D188" t="n">
+        <v>345260.7560583042</v>
+      </c>
+      <c r="E188" t="n">
+        <v>0</v>
+      </c>
+      <c r="F188" t="n">
+        <v>345559.6810604482</v>
+      </c>
+      <c r="G188" t="n">
+        <v>0</v>
+      </c>
+      <c r="H188" t="n">
+        <v>31344.87401919085</v>
+      </c>
+      <c r="I188" t="n">
+        <v>-16150749.97065179</v>
+      </c>
+      <c r="J188" t="n">
+        <v>0</v>
+      </c>
+      <c r="K188" t="n">
+        <v>0</v>
+      </c>
+      <c r="L188" t="n">
+        <v>42633726.82811298</v>
+      </c>
+      <c r="M188" t="n">
+        <v>26859881.41254083</v>
+      </c>
+      <c r="N188" t="n">
+        <v>213168.6341405648</v>
+      </c>
+      <c r="O188" t="n">
+        <v>0</v>
+      </c>
+      <c r="P188" t="n">
+        <v>213168.6341405648</v>
+      </c>
+      <c r="Q188" t="n">
+        <v>213168.6341405649</v>
+      </c>
+      <c r="R188" t="n">
+        <v>0</v>
+      </c>
+      <c r="S188" t="n">
+        <v>0</v>
+      </c>
+      <c r="T188" t="n">
+        <v>0</v>
+      </c>
+      <c r="U188" t="n">
+        <v>0</v>
+      </c>
+      <c r="V188" t="n">
+        <v>1.648000001907349</v>
+      </c>
+      <c r="W188" t="n">
+        <v>26859881.41254083</v>
+      </c>
+      <c r="X188" t="n">
+        <v>26859881.41254083</v>
+      </c>
+      <c r="Y188" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z188" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA188" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB188" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC188" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD188" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_200_el_price_150</t>
+        </is>
+      </c>
+      <c r="AE188" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\technology_selection\20260303191516_dh_0.5_ctax_200_el_price_150</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="n">
+        <v>21426076.2459629</v>
+      </c>
+      <c r="B189" t="n">
+        <v>298.9250021439932</v>
+      </c>
+      <c r="C189" t="n">
+        <v>0</v>
+      </c>
+      <c r="D189" t="n">
+        <v>345260.7560583042</v>
+      </c>
+      <c r="E189" t="n">
+        <v>0</v>
+      </c>
+      <c r="F189" t="n">
+        <v>345559.6810604482</v>
+      </c>
+      <c r="G189" t="n">
+        <v>0</v>
+      </c>
+      <c r="H189" t="n">
+        <v>258336.8895810759</v>
+      </c>
+      <c r="I189" t="n">
+        <v>-22021514.76718635</v>
+      </c>
+      <c r="J189" t="n">
+        <v>0</v>
+      </c>
+      <c r="K189" t="n">
+        <v>0</v>
+      </c>
+      <c r="L189" t="n">
+        <v>42843694.44250772</v>
+      </c>
+      <c r="M189" t="n">
+        <v>21426076.2459629</v>
+      </c>
+      <c r="N189" t="n">
+        <v>214218.4722125385</v>
+      </c>
+      <c r="O189" t="n">
+        <v>0</v>
+      </c>
+      <c r="P189" t="n">
+        <v>214218.4722125385</v>
+      </c>
+      <c r="Q189" t="n">
+        <v>214218.4722125386</v>
+      </c>
+      <c r="R189" t="n">
+        <v>0</v>
+      </c>
+      <c r="S189" t="n">
+        <v>0</v>
+      </c>
+      <c r="T189" t="n">
+        <v>0</v>
+      </c>
+      <c r="U189" t="n">
+        <v>0</v>
+      </c>
+      <c r="V189" t="n">
+        <v>1.526000022888184</v>
+      </c>
+      <c r="W189" t="n">
+        <v>21426076.24596276</v>
+      </c>
+      <c r="X189" t="n">
+        <v>21426076.2459629</v>
+      </c>
+      <c r="Y189" t="n">
+        <v>1.378357410430908e-07</v>
+      </c>
+      <c r="Z189" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA189" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB189" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC189" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD189" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_200_el_price_200</t>
+        </is>
+      </c>
+      <c r="AE189" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\technology_selection\20260303191706_dh_0.5_ctax_200_el_price_200</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="n">
+        <v>15829633.97238819</v>
+      </c>
+      <c r="B190" t="n">
+        <v>298.9250021439932</v>
+      </c>
+      <c r="C190" t="n">
+        <v>0</v>
+      </c>
+      <c r="D190" t="n">
+        <v>345260.7560583042</v>
+      </c>
+      <c r="E190" t="n">
+        <v>0</v>
+      </c>
+      <c r="F190" t="n">
+        <v>345559.6810604482</v>
+      </c>
+      <c r="G190" t="n">
+        <v>0</v>
+      </c>
+      <c r="H190" t="n">
+        <v>741276.9201512345</v>
+      </c>
+      <c r="I190" t="n">
+        <v>-28547616.59960862</v>
+      </c>
+      <c r="J190" t="n">
+        <v>0</v>
+      </c>
+      <c r="K190" t="n">
+        <v>0</v>
+      </c>
+      <c r="L190" t="n">
+        <v>43290413.97078513</v>
+      </c>
+      <c r="M190" t="n">
+        <v>15829633.97238819</v>
+      </c>
+      <c r="N190" t="n">
+        <v>216452.0698539255</v>
+      </c>
+      <c r="O190" t="n">
+        <v>0</v>
+      </c>
+      <c r="P190" t="n">
+        <v>216452.0698539255</v>
+      </c>
+      <c r="Q190" t="n">
+        <v>216452.0698539256</v>
+      </c>
+      <c r="R190" t="n">
+        <v>0</v>
+      </c>
+      <c r="S190" t="n">
+        <v>0</v>
+      </c>
+      <c r="T190" t="n">
+        <v>0</v>
+      </c>
+      <c r="U190" t="n">
+        <v>0</v>
+      </c>
+      <c r="V190" t="n">
+        <v>1.58899998664856</v>
+      </c>
+      <c r="W190" t="n">
+        <v>15829633.97238819</v>
+      </c>
+      <c r="X190" t="n">
+        <v>15829633.97238819</v>
+      </c>
+      <c r="Y190" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z190" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA190" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB190" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC190" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD190" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_200_el_price_250</t>
+        </is>
+      </c>
+      <c r="AE190" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\technology_selection\20260303191853_dh_0.5_ctax_200_el_price_250</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="n">
+        <v>10015193.2898675</v>
+      </c>
+      <c r="B191" t="n">
+        <v>298.9250021439932</v>
+      </c>
+      <c r="C191" t="n">
+        <v>0</v>
+      </c>
+      <c r="D191" t="n">
+        <v>345260.7560583042</v>
+      </c>
+      <c r="E191" t="n">
+        <v>0</v>
+      </c>
+      <c r="F191" t="n">
+        <v>345559.6810604482</v>
+      </c>
+      <c r="G191" t="n">
+        <v>0</v>
+      </c>
+      <c r="H191" t="n">
+        <v>1355408.143731272</v>
+      </c>
+      <c r="I191" t="n">
+        <v>-35544259.88752087</v>
+      </c>
+      <c r="J191" t="n">
+        <v>0</v>
+      </c>
+      <c r="K191" t="n">
+        <v>0</v>
+      </c>
+      <c r="L191" t="n">
+        <v>43858485.35259665</v>
+      </c>
+      <c r="M191" t="n">
+        <v>10015193.2898675</v>
+      </c>
+      <c r="N191" t="n">
+        <v>219292.4267629832</v>
+      </c>
+      <c r="O191" t="n">
+        <v>0</v>
+      </c>
+      <c r="P191" t="n">
+        <v>219292.4267629832</v>
+      </c>
+      <c r="Q191" t="n">
+        <v>219292.4267629832</v>
+      </c>
+      <c r="R191" t="n">
+        <v>0</v>
+      </c>
+      <c r="S191" t="n">
+        <v>0</v>
+      </c>
+      <c r="T191" t="n">
+        <v>0</v>
+      </c>
+      <c r="U191" t="n">
+        <v>0</v>
+      </c>
+      <c r="V191" t="n">
+        <v>1.546999931335449</v>
+      </c>
+      <c r="W191" t="n">
+        <v>10015193.28986724</v>
+      </c>
+      <c r="X191" t="n">
+        <v>10015193.2898675</v>
+      </c>
+      <c r="Y191" t="n">
+        <v>2.60770320892334e-07</v>
+      </c>
+      <c r="Z191" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA191" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB191" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC191" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD191" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_200_el_price_300</t>
+        </is>
+      </c>
+      <c r="AE191" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\technology_selection\20260303192042_dh_0.5_ctax_200_el_price_300</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="n">
+        <v>4016596.377110831</v>
+      </c>
+      <c r="B192" t="n">
+        <v>298.9250021439932</v>
+      </c>
+      <c r="C192" t="n">
+        <v>0</v>
+      </c>
+      <c r="D192" t="n">
+        <v>345260.7560583042</v>
+      </c>
+      <c r="E192" t="n">
+        <v>0</v>
+      </c>
+      <c r="F192" t="n">
+        <v>345559.6810604482</v>
+      </c>
+      <c r="G192" t="n">
+        <v>0</v>
+      </c>
+      <c r="H192" t="n">
+        <v>1785665.021901865</v>
+      </c>
+      <c r="I192" t="n">
+        <v>-42371101.29075594</v>
+      </c>
+      <c r="J192" t="n">
+        <v>0</v>
+      </c>
+      <c r="K192" t="n">
+        <v>0</v>
+      </c>
+      <c r="L192" t="n">
+        <v>44256472.96490446</v>
+      </c>
+      <c r="M192" t="n">
+        <v>4016596.377110831</v>
+      </c>
+      <c r="N192" t="n">
+        <v>221282.3648245222</v>
+      </c>
+      <c r="O192" t="n">
+        <v>0</v>
+      </c>
+      <c r="P192" t="n">
+        <v>221282.3648245222</v>
+      </c>
+      <c r="Q192" t="n">
+        <v>221282.3648245222</v>
+      </c>
+      <c r="R192" t="n">
+        <v>0</v>
+      </c>
+      <c r="S192" t="n">
+        <v>0</v>
+      </c>
+      <c r="T192" t="n">
+        <v>0</v>
+      </c>
+      <c r="U192" t="n">
+        <v>0</v>
+      </c>
+      <c r="V192" t="n">
+        <v>1.651999950408936</v>
+      </c>
+      <c r="W192" t="n">
+        <v>4016596.377110831</v>
+      </c>
+      <c r="X192" t="n">
+        <v>4016596.377110831</v>
+      </c>
+      <c r="Y192" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z192" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA192" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB192" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC192" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD192" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_200_el_price_350</t>
+        </is>
+      </c>
+      <c r="AE192" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\technology_selection\20260303192429_dh_0.5_ctax_200_el_price_350</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="n">
+        <v>-2062051.013089806</v>
+      </c>
+      <c r="B193" t="n">
+        <v>298.9250021439932</v>
+      </c>
+      <c r="C193" t="n">
+        <v>0</v>
+      </c>
+      <c r="D193" t="n">
+        <v>345260.7560583042</v>
+      </c>
+      <c r="E193" t="n">
+        <v>0</v>
+      </c>
+      <c r="F193" t="n">
+        <v>345559.6810604482</v>
+      </c>
+      <c r="G193" t="n">
+        <v>0</v>
+      </c>
+      <c r="H193" t="n">
+        <v>1953601.967314534</v>
+      </c>
+      <c r="I193" t="n">
+        <v>-48773027.30087596</v>
+      </c>
+      <c r="J193" t="n">
+        <v>0</v>
+      </c>
+      <c r="K193" t="n">
+        <v>0</v>
+      </c>
+      <c r="L193" t="n">
+        <v>44411814.63941117</v>
+      </c>
+      <c r="M193" t="n">
+        <v>-2062051.013089806</v>
+      </c>
+      <c r="N193" t="n">
+        <v>222059.0731970558</v>
+      </c>
+      <c r="O193" t="n">
+        <v>0</v>
+      </c>
+      <c r="P193" t="n">
+        <v>222059.0731970558</v>
+      </c>
+      <c r="Q193" t="n">
+        <v>222059.0731970558</v>
+      </c>
+      <c r="R193" t="n">
+        <v>0</v>
+      </c>
+      <c r="S193" t="n">
+        <v>0</v>
+      </c>
+      <c r="T193" t="n">
+        <v>0</v>
+      </c>
+      <c r="U193" t="n">
+        <v>0</v>
+      </c>
+      <c r="V193" t="n">
+        <v>1.523000001907349</v>
+      </c>
+      <c r="W193" t="n">
+        <v>-2062051.013089807</v>
+      </c>
+      <c r="X193" t="n">
+        <v>-2062051.013089806</v>
+      </c>
+      <c r="Y193" t="n">
+        <v>9.313225746154785e-10</v>
+      </c>
+      <c r="Z193" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA193" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB193" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC193" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD193" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_200_el_price_400</t>
+        </is>
+      </c>
+      <c r="AE193" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\technology_selection\20260303192616_dh_0.5_ctax_200_el_price_400</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="n">
+        <v>48241934.76623576</v>
+      </c>
+      <c r="B194" t="n">
+        <v>298.9250021439932</v>
+      </c>
+      <c r="C194" t="n">
+        <v>0</v>
+      </c>
+      <c r="D194" t="n">
+        <v>345260.7560583042</v>
+      </c>
+      <c r="E194" t="n">
+        <v>0</v>
+      </c>
+      <c r="F194" t="n">
+        <v>345559.6810604482</v>
+      </c>
+      <c r="G194" t="n">
+        <v>0</v>
+      </c>
+      <c r="H194" t="n">
+        <v>155.0546472912404</v>
+      </c>
+      <c r="I194" t="n">
+        <v>-5359875.275964418</v>
+      </c>
+      <c r="J194" t="n">
+        <v>0</v>
+      </c>
+      <c r="K194" t="n">
+        <v>0</v>
+      </c>
+      <c r="L194" t="n">
+        <v>53256095.30649244</v>
+      </c>
+      <c r="M194" t="n">
+        <v>48241934.76623576</v>
+      </c>
+      <c r="N194" t="n">
+        <v>213024.3812259698</v>
+      </c>
+      <c r="O194" t="n">
+        <v>0</v>
+      </c>
+      <c r="P194" t="n">
+        <v>213024.3812259698</v>
+      </c>
+      <c r="Q194" t="n">
+        <v>213024.3812259698</v>
+      </c>
+      <c r="R194" t="n">
+        <v>0</v>
+      </c>
+      <c r="S194" t="n">
+        <v>0</v>
+      </c>
+      <c r="T194" t="n">
+        <v>0</v>
+      </c>
+      <c r="U194" t="n">
+        <v>0</v>
+      </c>
+      <c r="V194" t="n">
+        <v>1.529999971389771</v>
+      </c>
+      <c r="W194" t="n">
+        <v>48241934.7662353</v>
+      </c>
+      <c r="X194" t="n">
+        <v>48241934.76623576</v>
+      </c>
+      <c r="Y194" t="n">
+        <v>4.619359970092773e-07</v>
+      </c>
+      <c r="Z194" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA194" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB194" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC194" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD194" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_250_el_price_50</t>
+        </is>
+      </c>
+      <c r="AE194" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\technology_selection\20260303192803_dh_0.5_ctax_250_el_price_50</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="n">
+        <v>42882059.49027134</v>
+      </c>
+      <c r="B195" t="n">
+        <v>298.9250021439932</v>
+      </c>
+      <c r="C195" t="n">
+        <v>0</v>
+      </c>
+      <c r="D195" t="n">
+        <v>345260.7560583042</v>
+      </c>
+      <c r="E195" t="n">
+        <v>0</v>
+      </c>
+      <c r="F195" t="n">
+        <v>345559.6810604482</v>
+      </c>
+      <c r="G195" t="n">
+        <v>0</v>
+      </c>
+      <c r="H195" t="n">
+        <v>155.0546472912404</v>
+      </c>
+      <c r="I195" t="n">
+        <v>-10719750.55192884</v>
+      </c>
+      <c r="J195" t="n">
+        <v>0</v>
+      </c>
+      <c r="K195" t="n">
+        <v>0</v>
+      </c>
+      <c r="L195" t="n">
+        <v>53256095.30649244</v>
+      </c>
+      <c r="M195" t="n">
+        <v>42882059.49027134</v>
+      </c>
+      <c r="N195" t="n">
+        <v>213024.3812259698</v>
+      </c>
+      <c r="O195" t="n">
+        <v>0</v>
+      </c>
+      <c r="P195" t="n">
+        <v>213024.3812259698</v>
+      </c>
+      <c r="Q195" t="n">
+        <v>213024.3812259698</v>
+      </c>
+      <c r="R195" t="n">
+        <v>0</v>
+      </c>
+      <c r="S195" t="n">
+        <v>0</v>
+      </c>
+      <c r="T195" t="n">
+        <v>0</v>
+      </c>
+      <c r="U195" t="n">
+        <v>0</v>
+      </c>
+      <c r="V195" t="n">
+        <v>1.523000001907349</v>
+      </c>
+      <c r="W195" t="n">
+        <v>42882059.49027134</v>
+      </c>
+      <c r="X195" t="n">
+        <v>42882059.49027134</v>
+      </c>
+      <c r="Y195" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z195" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA195" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB195" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC195" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD195" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_250_el_price_100</t>
+        </is>
+      </c>
+      <c r="AE195" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\technology_selection\20260303192950_dh_0.5_ctax_250_el_price_100</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="n">
+        <v>37516744.16002905</v>
+      </c>
+      <c r="B196" t="n">
+        <v>298.9250021439932</v>
+      </c>
+      <c r="C196" t="n">
+        <v>0</v>
+      </c>
+      <c r="D196" t="n">
+        <v>345260.7560583042</v>
+      </c>
+      <c r="E196" t="n">
+        <v>0</v>
+      </c>
+      <c r="F196" t="n">
+        <v>345559.6810604482</v>
+      </c>
+      <c r="G196" t="n">
+        <v>0</v>
+      </c>
+      <c r="H196" t="n">
+        <v>17022.10600403212</v>
+      </c>
+      <c r="I196" t="n">
+        <v>-16121435.4616591</v>
+      </c>
+      <c r="J196" t="n">
+        <v>0</v>
+      </c>
+      <c r="K196" t="n">
+        <v>0</v>
+      </c>
+      <c r="L196" t="n">
+        <v>53275597.83462367</v>
+      </c>
+      <c r="M196" t="n">
+        <v>37516744.16002905</v>
+      </c>
+      <c r="N196" t="n">
+        <v>213102.3913384947</v>
+      </c>
+      <c r="O196" t="n">
+        <v>0</v>
+      </c>
+      <c r="P196" t="n">
+        <v>213102.3913384947</v>
+      </c>
+      <c r="Q196" t="n">
+        <v>213102.3913384947</v>
+      </c>
+      <c r="R196" t="n">
+        <v>0</v>
+      </c>
+      <c r="S196" t="n">
+        <v>0</v>
+      </c>
+      <c r="T196" t="n">
+        <v>0</v>
+      </c>
+      <c r="U196" t="n">
+        <v>0</v>
+      </c>
+      <c r="V196" t="n">
+        <v>1.559999942779541</v>
+      </c>
+      <c r="W196" t="n">
+        <v>37516744.16002876</v>
+      </c>
+      <c r="X196" t="n">
+        <v>37516744.16002905</v>
+      </c>
+      <c r="Y196" t="n">
+        <v>2.905726432800293e-07</v>
+      </c>
+      <c r="Z196" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA196" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB196" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC196" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD196" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_250_el_price_150</t>
+        </is>
+      </c>
+      <c r="AE196" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\technology_selection\20260303193137_dh_0.5_ctax_250_el_price_150</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="n">
+        <v>32121607.49167487</v>
+      </c>
+      <c r="B197" t="n">
+        <v>298.9250021439932</v>
+      </c>
+      <c r="C197" t="n">
+        <v>0</v>
+      </c>
+      <c r="D197" t="n">
+        <v>345260.7560583042</v>
+      </c>
+      <c r="E197" t="n">
+        <v>0</v>
+      </c>
+      <c r="F197" t="n">
+        <v>345559.6810604482</v>
+      </c>
+      <c r="G197" t="n">
+        <v>0</v>
+      </c>
+      <c r="H197" t="n">
+        <v>124767.6003512254</v>
+      </c>
+      <c r="I197" t="n">
+        <v>-21748898.35219942</v>
+      </c>
+      <c r="J197" t="n">
+        <v>0</v>
+      </c>
+      <c r="K197" t="n">
+        <v>0</v>
+      </c>
+      <c r="L197" t="n">
+        <v>53400178.56246262</v>
+      </c>
+      <c r="M197" t="n">
+        <v>32121607.49167487</v>
+      </c>
+      <c r="N197" t="n">
+        <v>213600.7142498505</v>
+      </c>
+      <c r="O197" t="n">
+        <v>0</v>
+      </c>
+      <c r="P197" t="n">
+        <v>213600.7142498505</v>
+      </c>
+      <c r="Q197" t="n">
+        <v>213600.7142498505</v>
+      </c>
+      <c r="R197" t="n">
+        <v>0</v>
+      </c>
+      <c r="S197" t="n">
+        <v>0</v>
+      </c>
+      <c r="T197" t="n">
+        <v>0</v>
+      </c>
+      <c r="U197" t="n">
+        <v>0</v>
+      </c>
+      <c r="V197" t="n">
+        <v>1.553999900817871</v>
+      </c>
+      <c r="W197" t="n">
+        <v>32121607.49167449</v>
+      </c>
+      <c r="X197" t="n">
+        <v>32121607.49167487</v>
+      </c>
+      <c r="Y197" t="n">
+        <v>3.874301910400391e-07</v>
+      </c>
+      <c r="Z197" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA197" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB197" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC197" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD197" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_250_el_price_200</t>
+        </is>
+      </c>
+      <c r="AE197" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\technology_selection\20260303193550_dh_0.5_ctax_250_el_price_200</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="n">
+        <v>26612206.66289517</v>
+      </c>
+      <c r="B198" t="n">
+        <v>298.9250021439932</v>
+      </c>
+      <c r="C198" t="n">
+        <v>0</v>
+      </c>
+      <c r="D198" t="n">
+        <v>345260.7560583042</v>
+      </c>
+      <c r="E198" t="n">
+        <v>0</v>
+      </c>
+      <c r="F198" t="n">
+        <v>345559.6810604482</v>
+      </c>
+      <c r="G198" t="n">
+        <v>0</v>
+      </c>
+      <c r="H198" t="n">
+        <v>432120.8995392584</v>
+      </c>
+      <c r="I198" t="n">
+        <v>-27921029.73235332</v>
+      </c>
+      <c r="J198" t="n">
+        <v>0</v>
+      </c>
+      <c r="K198" t="n">
+        <v>0</v>
+      </c>
+      <c r="L198" t="n">
+        <v>53755555.81464878</v>
+      </c>
+      <c r="M198" t="n">
+        <v>26612206.66289517</v>
+      </c>
+      <c r="N198" t="n">
+        <v>215022.2232585951</v>
+      </c>
+      <c r="O198" t="n">
+        <v>0</v>
+      </c>
+      <c r="P198" t="n">
+        <v>215022.2232585951</v>
+      </c>
+      <c r="Q198" t="n">
+        <v>215022.2232585952</v>
+      </c>
+      <c r="R198" t="n">
+        <v>0</v>
+      </c>
+      <c r="S198" t="n">
+        <v>0</v>
+      </c>
+      <c r="T198" t="n">
+        <v>0</v>
+      </c>
+      <c r="U198" t="n">
+        <v>0</v>
+      </c>
+      <c r="V198" t="n">
+        <v>1.556999921798706</v>
+      </c>
+      <c r="W198" t="n">
+        <v>26612206.66289499</v>
+      </c>
+      <c r="X198" t="n">
+        <v>26612206.66289517</v>
+      </c>
+      <c r="Y198" t="n">
+        <v>1.825392246246338e-07</v>
+      </c>
+      <c r="Z198" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA198" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB198" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC198" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD198" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_250_el_price_250</t>
+        </is>
+      </c>
+      <c r="AE198" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\technology_selection\20260303193737_dh_0.5_ctax_250_el_price_250</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="n">
+        <v>20928591.1067262</v>
+      </c>
+      <c r="B199" t="n">
+        <v>298.9250021439932</v>
+      </c>
+      <c r="C199" t="n">
+        <v>0</v>
+      </c>
+      <c r="D199" t="n">
+        <v>345260.7560583042</v>
+      </c>
+      <c r="E199" t="n">
+        <v>0</v>
+      </c>
+      <c r="F199" t="n">
+        <v>345559.6810604482</v>
+      </c>
+      <c r="G199" t="n">
+        <v>0</v>
+      </c>
+      <c r="H199" t="n">
+        <v>925534.8617191213</v>
+      </c>
+      <c r="I199" t="n">
+        <v>-34668569.14447261</v>
+      </c>
+      <c r="J199" t="n">
+        <v>0</v>
+      </c>
+      <c r="K199" t="n">
+        <v>0</v>
+      </c>
+      <c r="L199" t="n">
+        <v>54326065.70841925</v>
+      </c>
+      <c r="M199" t="n">
+        <v>20928591.1067262</v>
+      </c>
+      <c r="N199" t="n">
+        <v>217304.262833677</v>
+      </c>
+      <c r="O199" t="n">
+        <v>0</v>
+      </c>
+      <c r="P199" t="n">
+        <v>217304.262833677</v>
+      </c>
+      <c r="Q199" t="n">
+        <v>217304.262833677</v>
+      </c>
+      <c r="R199" t="n">
+        <v>0</v>
+      </c>
+      <c r="S199" t="n">
+        <v>0</v>
+      </c>
+      <c r="T199" t="n">
+        <v>0</v>
+      </c>
+      <c r="U199" t="n">
+        <v>0</v>
+      </c>
+      <c r="V199" t="n">
+        <v>1.657000064849854</v>
+      </c>
+      <c r="W199" t="n">
+        <v>20928591.10672571</v>
+      </c>
+      <c r="X199" t="n">
+        <v>20928591.1067262</v>
+      </c>
+      <c r="Y199" t="n">
+        <v>4.954636096954346e-07</v>
+      </c>
+      <c r="Z199" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA199" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB199" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC199" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD199" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_250_el_price_300</t>
+        </is>
+      </c>
+      <c r="AE199" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\technology_selection\20260303193923_dh_0.5_ctax_250_el_price_300</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="n">
+        <v>15048394.76819916</v>
+      </c>
+      <c r="B200" t="n">
+        <v>298.9250021439932</v>
+      </c>
+      <c r="C200" t="n">
+        <v>0</v>
+      </c>
+      <c r="D200" t="n">
+        <v>345260.7560583042</v>
+      </c>
+      <c r="E200" t="n">
+        <v>0</v>
+      </c>
+      <c r="F200" t="n">
+        <v>345559.6810604482</v>
+      </c>
+      <c r="G200" t="n">
+        <v>0</v>
+      </c>
+      <c r="H200" t="n">
+        <v>1516134.934118922</v>
+      </c>
+      <c r="I200" t="n">
+        <v>-41822246.88911173</v>
+      </c>
+      <c r="J200" t="n">
+        <v>0</v>
+      </c>
+      <c r="K200" t="n">
+        <v>0</v>
+      </c>
+      <c r="L200" t="n">
+        <v>55008947.04213152</v>
+      </c>
+      <c r="M200" t="n">
+        <v>15048394.76819916</v>
+      </c>
+      <c r="N200" t="n">
+        <v>220035.7881685261</v>
+      </c>
+      <c r="O200" t="n">
+        <v>0</v>
+      </c>
+      <c r="P200" t="n">
+        <v>220035.7881685261</v>
+      </c>
+      <c r="Q200" t="n">
+        <v>220035.7881685261</v>
+      </c>
+      <c r="R200" t="n">
+        <v>0</v>
+      </c>
+      <c r="S200" t="n">
+        <v>0</v>
+      </c>
+      <c r="T200" t="n">
+        <v>0</v>
+      </c>
+      <c r="U200" t="n">
+        <v>0</v>
+      </c>
+      <c r="V200" t="n">
+        <v>1.631999969482422</v>
+      </c>
+      <c r="W200" t="n">
+        <v>15048394.76819916</v>
+      </c>
+      <c r="X200" t="n">
+        <v>15048394.76819916</v>
+      </c>
+      <c r="Y200" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z200" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA200" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB200" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC200" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD200" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_250_el_price_350</t>
+        </is>
+      </c>
+      <c r="AE200" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\technology_selection\20260303194114_dh_0.5_ctax_250_el_price_350</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="n">
+        <v>9026728.141834624</v>
+      </c>
+      <c r="B201" t="n">
+        <v>298.9250021439932</v>
+      </c>
+      <c r="C201" t="n">
+        <v>0</v>
+      </c>
+      <c r="D201" t="n">
+        <v>345260.7560583042</v>
+      </c>
+      <c r="E201" t="n">
+        <v>0</v>
+      </c>
+      <c r="F201" t="n">
+        <v>345559.6810604482</v>
+      </c>
+      <c r="G201" t="n">
+        <v>0</v>
+      </c>
+      <c r="H201" t="n">
+        <v>1826239.049474173</v>
+      </c>
+      <c r="I201" t="n">
+        <v>-48512575.51421103</v>
+      </c>
+      <c r="J201" t="n">
+        <v>0</v>
+      </c>
+      <c r="K201" t="n">
+        <v>0</v>
+      </c>
+      <c r="L201" t="n">
+        <v>55367504.92551103</v>
+      </c>
+      <c r="M201" t="n">
+        <v>9026728.141834624</v>
+      </c>
+      <c r="N201" t="n">
+        <v>221470.0197020441</v>
+      </c>
+      <c r="O201" t="n">
+        <v>0</v>
+      </c>
+      <c r="P201" t="n">
+        <v>221470.0197020441</v>
+      </c>
+      <c r="Q201" t="n">
+        <v>221470.0197020441</v>
+      </c>
+      <c r="R201" t="n">
+        <v>0</v>
+      </c>
+      <c r="S201" t="n">
+        <v>0</v>
+      </c>
+      <c r="T201" t="n">
+        <v>0</v>
+      </c>
+      <c r="U201" t="n">
+        <v>0</v>
+      </c>
+      <c r="V201" t="n">
+        <v>1.555999994277954</v>
+      </c>
+      <c r="W201" t="n">
+        <v>9026728.14183452</v>
+      </c>
+      <c r="X201" t="n">
+        <v>9026728.141834624</v>
+      </c>
+      <c r="Y201" t="n">
+        <v>1.043081283569336e-07</v>
+      </c>
+      <c r="Z201" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA201" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB201" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC201" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD201" t="inlineStr">
+        <is>
+          <t>dh_0.5_ctax_250_el_price_400</t>
+        </is>
+      </c>
+      <c r="AE201" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_WtE\raw_results\technology_selection\20260303194302_dh_0.5_ctax_250_el_price_400</t>
         </is>
       </c>
     </row>

</xml_diff>